<commit_message>
for this module, northbank is replaced by udacibank to ensure that there is not even distant resemblance to the real company
</commit_message>
<xml_diff>
--- a/07_ai-security-metrics-and-dashboarding/exercises/solution/kri_definitions.xlsx
+++ b/07_ai-security-metrics-and-dashboarding/exercises/solution/kri_definitions.xlsx
@@ -537,7 +537,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NorthBank — Portfolio KRI Exercise</t>
+          <t>UdaciBank — Portfolio KRI Exercise</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>COMPANY: NorthBank (digital-only fintech, 850 employees, US + UK)</t>
+          <t>COMPANY: UdaciBank (digital-only fintech, 850 employees, US + UK)</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  R-03: Anomalous refusal-rate spikes on the assistant indicate either policy drift or attempted misuse — both warrant investigationant indicate prompt-injection / abuse.</t>
+          <t xml:space="preserve">  R-03: Anomalous behavior on the assistant — including refusal-rate spikes and jailbreak-classifier hits — indicates either policy drift or attempted misuse and warrants investigation.</t>
         </is>
       </c>
     </row>
@@ -837,45 +837,45 @@
       </c>
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>Refusal rate — LLM customer-support assistant (Aurora Assistant)</t>
+          <t>Jailbreak-classifier hit rate — Aurora Assistant (LLM customer-support)</t>
         </is>
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>R-03: Anomalous refusal-rate spikes on the assistant indicate either policy drift or attempted misuse — both warrant investigation</t>
+          <t>R-03: Anomalous behavior on the assistant (refusal-rate spikes + jailbreak-classifier hits) — policy drift or attempted misuse</t>
         </is>
       </c>
       <c r="D4" s="17" t="inlineStr">
         <is>
-          <t>LLM gateway turn log (data/refusal_log.csv-shaped fixture for SP7 demo): timestamp, session_id, model_version, turn_index, refusal_flag — rolling 24h aggregate.
-Reasoning: refusal_flag is already emitted by the gateway's policy classifier, so we don't need a new pipeline — only a daily aggregator.</t>
+          <t>LLM gateway turn log: `jailbreak_flag` column emitted inline by the policy/jailbreak classifier per turn. KRI = (turns flagged) / (total turns) over a rolling 7-day window.
+Reasoning: jailbreak_flag is already produced by the gateway classifier — no new pipeline needed; rolling 7-day window smooths over single-attempt noise while still catching coordinated probing campaigns.</t>
         </is>
       </c>
       <c r="E4" s="17" t="inlineStr">
         <is>
-          <t>green ≤ 3% / amber 3–7% / red &gt; 7% (rolling 24h refusal rate).
-Reasoning: &lt;3% matches Aurora's historical baseline (Q4 ops report); &gt;7% has only been hit during the two known prompt-injection campaigns last year.</t>
+          <t>green ≤ 0.05% / amber 0.05–0.20% / red &gt; 0.20% (rolling 7-day jailbreak hit rate).
+Reasoning: ≤0.05% matches Aurora's historical baseline of accidental classifier hits; &gt;0.20% has only been observed during known adversarial probing (Q1 2026 incident), so crossing it implies active misuse.</t>
         </is>
       </c>
       <c r="F4" s="17" t="inlineStr">
         <is>
-          <t>Daily (rolling 24h)</t>
+          <t>Daily (rolling 7-day window)</t>
         </is>
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>LLM Platform Lead</t>
+          <t>AppSec Lead</t>
         </is>
       </c>
       <c r="H4" s="17" t="inlineStr">
         <is>
-          <t>Platform Lead → AI Review Board at amber → CRO + AppSec at red.
-Reasoning: amber may be policy drift (own it on the platform team); red implies active misuse (needs CRO + AppSec eyes).</t>
+          <t>AppSec Lead → AI Review Board at amber → CISO + Legal at red.
+Reasoning: jailbreak attempts are adversarial by definition — AppSec owns first response; Legal needs an early heads-up in case incident-disclosure obligations get triggered.</t>
         </is>
       </c>
       <c r="I4" s="17" t="inlineStr">
         <is>
-          <t>Has the assistant started refusing more than usual — and if so, is it policy drift or someone probing for misuse?</t>
+          <t>How often is someone successfully provoking the assistant past its safeguards — and is the rate trending up?</t>
         </is>
       </c>
     </row>
@@ -1377,18 +1377,18 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>Refusal rate (Aurora Assistant)</t>
+          <t>Jailbreak-classifier hit rate (Aurora Assistant)</t>
         </is>
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>R-03: Anomalous refusal-rate spikes</t>
+          <t>R-03: Anomalous behavior on the assistant (refusal-rate spikes + jailbreak hits)</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
           <t>M-03 Aurora Assistant (primary).
-Reasoning: only one production LLM-powered customer surface today; if a second LLM goes live (e.g., dispute-summarization), this same KRI extends by adding a model_id filter on the gateway log.</t>
+Reasoning: today's only LLM-fronted customer surface; the same KRI extends to any future LLM (e.g., dispute-summarization assistant) by adding a model_id filter on the gateway log.</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>Refusal rate — Aurora Assistant</t>
+          <t>Jailbreak-classifier hit rate — Aurora Assistant</t>
         </is>
       </c>
       <c r="C4" s="16" t="inlineStr">
@@ -1565,12 +1565,12 @@
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>g ≤ 3% / a 3-7% / r &gt; 7%</t>
+          <t>g ≤ 0.05% / a 0.05-0.20% / r &gt; 0.20% (rolling 7-day)</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>Placeholder until the LLM-gateway turn-log pipe lands in the dashboard; design spec captures threshold (3% / 7%), 24h cadence, and Platform Lead → AIRB → CRO escalation so engineering can implement next sprint.</t>
+          <t>Placeholder until the LLM-gateway jailbreak-flag pipe lands in the dashboard; design spec captures threshold (0.05% / 0.20%), 7-day rolling cadence, and AppSec Lead → AIRB → CISO + Legal escalation so engineering can implement next sprint.</t>
         </is>
       </c>
     </row>

</xml_diff>